<commit_message>
docs: sync SPEC.md and Excel with current dashboard (remove bar chart references, add movement KPI)
</commit_message>
<xml_diff>
--- a/SPEC-v2.xlsx
+++ b/SPEC-v2.xlsx
@@ -1062,7 +1062,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>AC-DASH-002: Given monthly transactions exist, when the dashboard renders, then the revenue/expense bar chart shows data for the current year.</t>
+          <t>AC-DASH-002: Given income and expense transactions exist, when the dashboard renders, then the income vs. expenses totals pie chart shows both slices.</t>
         </is>
       </c>
     </row>
@@ -4532,7 +4532,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>The dashboard shall display KPI cards: total clients, total projects, active projects.</t>
+          <t>The dashboard shall display KPI cards: total clients, total projects, active projects, employees, and total movement.</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">

</xml_diff>